<commit_message>
Updated description, message, output variables and removed redundant tests.
</commit_message>
<xml_diff>
--- a/rules/CORE-000562/positive/02/data/unit-test-coreid-CG0273-positive 2.xlsx
+++ b/rules/CORE-000562/positive/02/data/unit-test-coreid-CG0273-positive 2.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1338,11 +1338,6 @@
       <c r="C20" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
           <t>HLTSUBJI</t>
@@ -1378,7 +1373,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>CDISCPILOT02</t>
+          <t>CDISCPILOT01</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1387,49 +1382,43 @@
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>HLTSUBJI</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Healthy Subject Indicator</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>C49488</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>2020-03-28</t>
+        <v>1</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>INDIC</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Trial Disease/Condition Indication</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Alzheimer's Disease (Disorder)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>26929004</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>SNOMED</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>2019-03-01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>CDISCPILOT03</t>
+          <t>CDISCPILOT01</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1438,40 +1427,34 @@
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>HLTSUBJI</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Healthy Subject Indicator</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>C49487</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>INTMODEL</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Intervention Model</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>PARALLEL</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>C82639</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>CDISC</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>
@@ -1493,32 +1476,32 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>INDIC</t>
+          <t>INTTYPE</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Trial Disease/Condition Indication</t>
+          <t>Intervention Type</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Alzheimer's Disease (Disorder)</t>
+          <t>DRUG</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>26929004</t>
+          <t>C1909</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>SNOMED</t>
+          <t>CDISC</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>2019-03-01</t>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -1538,32 +1521,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>INTMODEL</t>
+          <t>LENGTH</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Intervention Model</t>
+          <t>Trial Length</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>PARALLEL</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>C82639</t>
+          <t>P28W</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>ISO 8601</t>
         </is>
       </c>
     </row>
@@ -1583,32 +1556,17 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>INTTYPE</t>
+          <t>NARMS</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Intervention Type</t>
+          <t>Planned Number of Arms</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>DRUG</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>C1909</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1626,24 +1584,24 @@
       <c r="C26" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>EFFICACY</t>
+        </is>
+      </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>OBJPRIM</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Trial Length</t>
+          <t>Trial Primary Objective</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>P28W</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>ISO 8601</t>
+          <t>To document the efficacy profile of Zanomaline.</t>
         </is>
       </c>
     </row>
@@ -1659,21 +1617,26 @@
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>SAFETY</t>
+        </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>NARMS</t>
+          <t>OBJPRIM</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Planned Number of Arms</t>
+          <t>Trial Primary Objective</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>To document the safety profile of Zanomaline.</t>
         </is>
       </c>
     </row>
@@ -1698,17 +1661,17 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>OBJPRIM</t>
+          <t>OUTMSPRI</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Trial Primary Objective</t>
+          <t>Primary Outcome Measure</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>To document the efficacy profile of Zanomaline.</t>
+          <t>To assess the dose-dependent improvement in subject depression. Improved scores on the Patient Health Questionnaire(PHQ-9) and the Hamilton Depression Rating Scale(HAMD 17) will indicate improvements.</t>
         </is>
       </c>
     </row>
@@ -1728,22 +1691,22 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>SAFETY</t>
+          <t>EFFICACY</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>OBJPRIM</t>
+          <t>OUTMSPRI</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Trial Primary Objective</t>
+          <t>Primary Outcome Measure</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>To document the safety profile of Zanomaline.</t>
+          <t>To assess the dose-dependent improvements in satisfaction with subjects' lives as a whole. Improved scores on the Satisfaction With Life Survery (SWLS) will indicate improvements.</t>
         </is>
       </c>
     </row>
@@ -1758,8 +1721,10 @@
           <t>TS</t>
         </is>
       </c>
-      <c r="C30" s="5" t="n">
-        <v>1</v>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
@@ -1778,7 +1743,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>To assess the dose-dependent improvement in subject depression. Improved scores on the Patient Health Questionnaire(PHQ-9) and the Hamilton Depression Rating Scale(HAMD 17) will indicate improvements.</t>
+          <t>To assess the dose-dependent improvements in subject memory and learning. Improved scores on the Auditory Verbal Learning Test (AVLT-REY) will indicate improvements.</t>
         </is>
       </c>
     </row>
@@ -1793,12 +1758,14 @@
           <t>TS</t>
         </is>
       </c>
-      <c r="C31" s="5" t="n">
-        <v>2</v>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>EFFICACY</t>
+          <t>SAFETY</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1813,7 +1780,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>To assess the dose-dependent improvements in satisfaction with subjects' lives as a whole. Improved scores on the Satisfaction With Life Survery (SWLS) will indicate improvements.</t>
+          <t>Type, frequency, and severity of laboratory abnormalities</t>
         </is>
       </c>
     </row>
@@ -1830,12 +1797,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>EFFICACY</t>
+          <t>SAFETY</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1850,7 +1817,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>To assess the dose-dependent improvements in subject memory and learning. Improved scores on the Auditory Verbal Learning Test (AVLT-REY) will indicate improvements.</t>
+          <t>Type, frequency, and severity of adverse events (AEs)</t>
         </is>
       </c>
     </row>
@@ -1865,29 +1832,32 @@
           <t>TS</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>SAFETY</t>
-        </is>
+      <c r="C33" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>OUTMSPRI</t>
+          <t>PCLAS</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Primary Outcome Measure</t>
+          <t>Pharmacologic Class</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Type, frequency, and severity of laboratory abnormalities</t>
+          <t>Acetylcholine Release Inhibitor</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>N0000175771</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>MED-RT</t>
         </is>
       </c>
     </row>
@@ -1902,29 +1872,22 @@
           <t>TS</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>SAFETY</t>
-        </is>
+      <c r="C34" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>OUTMSPRI</t>
+          <t>PLANSUB</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Primary Outcome Measure</t>
+          <t>Planned Number of Subjects</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Type, frequency, and severity of adverse events (AEs)</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -1944,27 +1907,32 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>PCLAS</t>
+          <t>RANDOM</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Pharmacologic Class</t>
+          <t>Trial is Randomized</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Acetylcholine Release Inhibitor</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>N0000175771</t>
+          <t>C49488</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>MED-RT</t>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1952,17 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>PLANSUB</t>
+          <t>RANDQT</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Planned Number of Subjects</t>
+          <t>Randomization Quotient</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0.67</t>
         </is>
       </c>
     </row>
@@ -2014,32 +1982,27 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>RANDOM</t>
+          <t>REGID</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Trial is Randomized</t>
+          <t>Registry Identifier</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>NCT00000000</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>C49488</t>
+          <t>NCT00000000</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>clinicaltrials.gov</t>
         </is>
       </c>
     </row>
@@ -2059,17 +2022,32 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>RANDQT</t>
+          <t>ROUTE</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Randomization Quotient</t>
+          <t>Route of Administration</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>SUBCUTANEOUS</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>C38299</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -2089,27 +2067,17 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>REGID</t>
+          <t>SDTIGVER</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Registry Identifier</t>
+          <t>SDTM IG Version</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>NCT00000000</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>NCT00000000</t>
-        </is>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>clinicaltrials.gov</t>
+          <t>3.3</t>
         </is>
       </c>
     </row>
@@ -2129,32 +2097,17 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>ROUTE</t>
+          <t>SDTMVER</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Route of Administration</t>
+          <t>SDTM Version</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>SUBCUTANEOUS</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>C38299</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>1.7</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2127,22 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>SDTIGVER</t>
+          <t>SENDTC</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>SDTM IG Version</t>
+          <t>Study End Date</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>2014-11-01</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>ISO 8601</t>
         </is>
       </c>
     </row>
@@ -2204,17 +2162,32 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>SDTMVER</t>
+          <t>SEXPOP</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>SDTM Version</t>
+          <t>Sex of Participants</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>C49636</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -2234,22 +2207,17 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>SENDTC</t>
+          <t>SPONSOR</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Study End Date</t>
+          <t>Clinical Study Sponsor</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>2014-11-01</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>ISO 8601</t>
+          <t>SDTM Metadata Submission Guidelines Team</t>
         </is>
       </c>
     </row>
@@ -2269,32 +2237,22 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>SEXPOP</t>
+          <t>SSTDTC</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Sex of Participants</t>
+          <t>Study Start Date</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>BOTH</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>C49636</t>
+          <t>2012-10-06</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K44" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>ISO 8601</t>
         </is>
       </c>
     </row>
@@ -2314,17 +2272,17 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>SPONSOR</t>
+          <t>STOPRULE</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Clinical Study Sponsor</t>
+          <t>Study Stop Rules</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>SDTM Metadata Submission Guidelines Team</t>
+          <t>NONE</t>
         </is>
       </c>
     </row>
@@ -2344,22 +2302,32 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>SSTDTC</t>
+          <t>STYPE</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Study Start Date</t>
+          <t>Study Type</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>2012-10-06</t>
+          <t>INTERVENTIONAL</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>C98388</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>ISO 8601</t>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -2379,17 +2347,32 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>STOPRULE</t>
+          <t>TBLIND</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Study Stop Rules</t>
+          <t>Trial Blinding Schema</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DOUBLE BLIND</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>C15228</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -2409,22 +2392,22 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>STYPE</t>
+          <t>TCNTRL</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Study Type</t>
+          <t>Control Type</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>INTERVENTIONAL</t>
+          <t>PLACEBO</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>C98388</t>
+          <t>C49648</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -2452,36 +2435,21 @@
       <c r="C49" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>TBLIND</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>Trial Blinding Schema</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>DOUBLE BLIND</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>C15228</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
-        </is>
-      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>TDIGRP</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Diagnosis Group</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="6" t="n"/>
+      <c r="K49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -2499,22 +2467,22 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>TCNTRL</t>
+          <t>TINDTP</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Control Type</t>
+          <t>Trial Intent Type</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>PLACEBO</t>
+          <t>TREATMENT</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>C49648</t>
+          <t>C49656</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -2542,60 +2510,66 @@
       <c r="C51" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>TDIGRP</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>Diagnosis Group</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="n"/>
-      <c r="H51" s="6" t="n"/>
-      <c r="I51" s="6" t="n"/>
-      <c r="J51" s="6" t="n"/>
-      <c r="K51" s="6" t="n"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>TITLE</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Trial Title</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Safety and Efficacy of Zanomaline in Patients with Mild to Moderate Alzheimers Disease.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
           <t>TS</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>TDIGRP</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>Diagnosis Group</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>Alzheimer's Disease (Disorder)</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="n"/>
-      <c r="I52" s="6" t="n"/>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="6" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>TPHASE</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Trial Phase Classification</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>PHASE II TRIAL</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>C15601</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -2613,32 +2587,27 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>TINDTP</t>
+          <t>TRT</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Trial Intent Type</t>
+          <t>Investigational Therapy or Treatment</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>TREATMENT</t>
+          <t>Zanomaline</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>C49656</t>
+          <t>0XXX0X00XX</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K53" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
+          <t>UNII</t>
         </is>
       </c>
     </row>
@@ -2658,17 +2627,32 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>TITLE</t>
+          <t>TTYPE</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Trial Title</t>
+          <t>Trial Type</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Safety and Efficacy of Zanomaline in Patients with Mild to Moderate Alzheimers Disease.</t>
+          <t>SAFETY</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>C49667</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>CDISC</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>2020-03-27</t>
         </is>
       </c>
     </row>
@@ -2683,27 +2667,29 @@
           <t>TS</t>
         </is>
       </c>
-      <c r="C55" s="5" t="n">
-        <v>1</v>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>TPHASE</t>
+          <t>TTYPE</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Trial Phase Classification</t>
+          <t>Trial Type</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>PHASE II TRIAL</t>
+          <t>EFFICACY</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>C15601</t>
+          <t>C49666</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -2712,138 +2698,6 @@
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>CDISCPILOT01</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>TS</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>TRT</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>Investigational Therapy or Treatment</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>Zanomaline</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>0XXX0X00XX</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>UNII</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>CDISCPILOT01</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>TS</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>TTYPE</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>Trial Type</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
-        <is>
-          <t>SAFETY</t>
-        </is>
-      </c>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>C49667</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K57" s="5" t="inlineStr">
-        <is>
-          <t>2020-03-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>CDISCPILOT01</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>TS</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>TTYPE</t>
-        </is>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>Trial Type</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>EFFICACY</t>
-        </is>
-      </c>
-      <c r="I58" s="5" t="inlineStr">
-        <is>
-          <t>C49666</t>
-        </is>
-      </c>
-      <c r="J58" s="5" t="inlineStr">
-        <is>
-          <t>CDISC</t>
-        </is>
-      </c>
-      <c r="K58" s="5" t="inlineStr">
         <is>
           <t>2020-03-27</t>
         </is>

</xml_diff>